<commit_message>
otptool: add export command for OTP raw image to JSONC format
1. Add export command for OTP raw image to JSONC format.
2. Rename excel_to_json.py tool.
3. Update AST2700A2 memory map.
4. Update README for new export command.

Signed-off-by: Neal Liu <neal_liu@aspeedtech.com>
Change-Id: I9fee28dbfc89220d3a63475bd35764c7c0bfe754
</commit_message>
<xml_diff>
--- a/tools/memory_map/AST2700A2_OTP_memory_map.xlsx
+++ b/tools/memory_map/AST2700A2_OTP_memory_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sdk\ast2700\OTP\memory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F5F94B1-81B8-4B40-8384-4B9580233212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B28EE68B-5E3E-4F1E-906C-B9764394DDB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{40652B66-A45B-48BE-91E6-4A13E915CABA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="7" xr2:uid="{40652B66-A45B-48BE-91E6-4A13E915CABA}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="6" r:id="rId1"/>
@@ -3623,7 +3623,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4077,29 +4077,23 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -4504,13 +4498,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="151" t="s">
+      <c r="A1" s="156" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="151"/>
-      <c r="C1" s="151"/>
-      <c r="D1" s="151"/>
-      <c r="E1" s="151"/>
+      <c r="B1" s="156"/>
+      <c r="C1" s="156"/>
+      <c r="D1" s="156"/>
+      <c r="E1" s="156"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="125" t="s">
@@ -7440,10 +7434,10 @@
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="152" t="s">
+      <c r="A61" s="151" t="s">
         <v>356</v>
       </c>
-      <c r="B61" s="153" t="s">
+      <c r="B61" s="152" t="s">
         <v>26</v>
       </c>
       <c r="C61" s="102" t="s">
@@ -7463,10 +7457,10 @@
       <c r="G61" s="104" t="s">
         <v>25</v>
       </c>
-      <c r="H61" s="157" t="s">
+      <c r="H61" s="154" t="s">
         <v>684</v>
       </c>
-      <c r="I61" s="158" t="s">
+      <c r="I61" s="155" t="s">
         <v>392</v>
       </c>
     </row>
@@ -7477,7 +7471,7 @@
       <c r="B62" s="29" t="s">
         <v>698</v>
       </c>
-      <c r="C62" s="154">
+      <c r="C62" s="64">
         <v>7</v>
       </c>
       <c r="D62" s="16">
@@ -7508,7 +7502,7 @@
       <c r="B63" s="29" t="s">
         <v>699</v>
       </c>
-      <c r="C63" s="154">
+      <c r="C63" s="64">
         <v>6</v>
       </c>
       <c r="D63" s="16">
@@ -7539,7 +7533,7 @@
       <c r="B64" s="29" t="s">
         <v>700</v>
       </c>
-      <c r="C64" s="154">
+      <c r="C64" s="64">
         <v>5</v>
       </c>
       <c r="D64" s="16">
@@ -7570,7 +7564,7 @@
       <c r="B65" s="29" t="s">
         <v>701</v>
       </c>
-      <c r="C65" s="154">
+      <c r="C65" s="64">
         <v>4</v>
       </c>
       <c r="D65" s="16">
@@ -7601,7 +7595,7 @@
       <c r="B66" s="29" t="s">
         <v>702</v>
       </c>
-      <c r="C66" s="154">
+      <c r="C66" s="64">
         <v>3</v>
       </c>
       <c r="D66" s="16">
@@ -7632,7 +7626,7 @@
       <c r="B67" s="29" t="s">
         <v>703</v>
       </c>
-      <c r="C67" s="154">
+      <c r="C67" s="64">
         <v>2</v>
       </c>
       <c r="D67" s="16">
@@ -7663,7 +7657,7 @@
       <c r="B68" s="29" t="s">
         <v>704</v>
       </c>
-      <c r="C68" s="154">
+      <c r="C68" s="64">
         <v>1</v>
       </c>
       <c r="D68" s="16">
@@ -7691,10 +7685,10 @@
       <c r="A69" s="122" t="s">
         <v>356</v>
       </c>
-      <c r="B69" s="155" t="s">
+      <c r="B69" s="153" t="s">
         <v>705</v>
       </c>
-      <c r="C69" s="156">
+      <c r="C69" s="95">
         <v>0</v>
       </c>
       <c r="D69" s="66">
@@ -14773,7 +14767,7 @@
         <v>587</v>
       </c>
       <c r="C39" s="96" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="D39" s="59">
         <v>256</v>
@@ -14802,7 +14796,7 @@
         <v>588</v>
       </c>
       <c r="C40" s="96" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="D40" s="59">
         <v>256</v>
@@ -14831,7 +14825,7 @@
         <v>589</v>
       </c>
       <c r="C41" s="96" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="D41" s="59">
         <v>256</v>
@@ -14860,7 +14854,7 @@
         <v>590</v>
       </c>
       <c r="C42" s="96" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="D42" s="59">
         <v>256</v>
@@ -15301,6 +15295,34 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="0358a91d-8923-4300-9035-92feb74d70aa">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="94916c3f-a887-466e-9071-419f2f5fc067" xsi:nil="true"/>
+    <TaxCatchAll xmlns="0358a91d-8923-4300-9035-92feb74d70aa" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="94916c3f-a887-466e-9071-419f2f5fc067">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB031FF8E1109D43B2BDF0F43F684A4E" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b896ebdbfa452e7a07541eac816e2062">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="94916c3f-a887-466e-9071-419f2f5fc067" xmlns:ns3="0358a91d-8923-4300-9035-92feb74d70aa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="556acc82b7336cf142ff4903a3ab7ecb" ns2:_="" ns3:_="">
     <xsd:import namespace="94916c3f-a887-466e-9071-419f2f5fc067"/>
@@ -15555,49 +15577,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="0358a91d-8923-4300-9035-92feb74d70aa">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="94916c3f-a887-466e-9071-419f2f5fc067" xsi:nil="true"/>
-    <TaxCatchAll xmlns="0358a91d-8923-4300-9035-92feb74d70aa" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="94916c3f-a887-466e-9071-419f2f5fc067">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AAF0E9-722A-46AD-84E0-1D9BE67AFFE4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06808489-AD29-49EF-A920-5725306266D8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="94916c3f-a887-466e-9071-419f2f5fc067"/>
-    <ds:schemaRef ds:uri="0358a91d-8923-4300-9035-92feb74d70aa"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -15620,9 +15603,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06808489-AD29-49EF-A920-5725306266D8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AAF0E9-722A-46AD-84E0-1D9BE67AFFE4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="94916c3f-a887-466e-9071-419f2f5fc067"/>
+    <ds:schemaRef ds:uri="0358a91d-8923-4300-9035-92feb74d70aa"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
otp: update AST2700-A2 OTP fields to memory map v2.3
Sync socsec's OTP field definitions with the AST2700-A2 v2.3 memory
map:

- Add retire_mechanism_option (OTPCFG0[8]): selects the key
  retirement policy, i.e. whether a key can only retire itself or can
  also retire other key IDs via the OTPRBP retire bits (OTPRBP0/1/3).
- Remove SoC_FMC_Hardware_SVN_0~3 from the OTPRBP region, no longer
  defined in v2.3 of the memory map.
- Update tools/memory_map/AST2700A2_OTP_memory_map.xlsx and
  tools/samples/sample_2700_A2.jsonc to match the above.
- Note the pandas/openpyxl dependencies required by
  scripts/excel_to_json.py in tools/README.md.

Signed-off-by: jheng-shuo_lin <jheng-shuo_lin@aspeedtech.com>
Change-Id: Ibbd36f44bd55eb9ba1add07f60457f286df24e71
</commit_message>
<xml_diff>
--- a/tools/memory_map/AST2700A2_OTP_memory_map.xlsx
+++ b/tools/memory_map/AST2700A2_OTP_memory_map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sdk\ast2700\OTP\memory\release\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\jheng-shuo_lin\socsec\tools\memory_map\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{215BF77B-7B06-46F4-8AFC-7FA2981CDB3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{467A2A65-08A1-4196-B498-038062358232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{40652B66-A45B-48BE-91E6-4A13E915CABA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{40652B66-A45B-48BE-91E6-4A13E915CABA}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="6" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1468" uniqueCount="733">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1466" uniqueCount="734">
   <si>
     <t>High Level overview of OTP memory layout</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2862,10 +2862,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>SoC FMC Hardware SVN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>dis_cptra_owner_key_retry</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -2889,14 +2885,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>SoC FMC hardware SVN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>47: 0</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Disable OTP Memory Factory Test Mode
 0: enable
 1: disable
@@ -2984,10 +2972,6 @@
   <si>
     <t>The blue color fields show what would be provisioned by ASPEED.
 OTPROM, OTPCFG, OTPSTRAP, OTPCAL, OTPPUF</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>v2p1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -3054,6 +3038,29 @@
   </si>
   <si>
     <t>800</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v2p3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>175: 0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>15:4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>retire_mechanism_option</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enable key retirement mechanism option 
+0: can only retire itself key #id
+1: can retire others key #id except itself
+There are some key retire bits in OTPRBP region (ex: OTPRBP0/1/3) used of be programmed if the keys need of be retired. This option chooses the retire mechanism policy for different use cases.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -4233,6 +4240,24 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4244,24 +4269,6 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -4666,20 +4673,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="162" t="s">
+      <c r="A1" s="168" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="162"/>
-      <c r="C1" s="162"/>
-      <c r="D1" s="162"/>
-      <c r="E1" s="162"/>
+      <c r="B1" s="168"/>
+      <c r="C1" s="168"/>
+      <c r="D1" s="168"/>
+      <c r="E1" s="168"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="124" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="125" t="s">
-        <v>722</v>
+        <v>729</v>
       </c>
       <c r="C2" s="48"/>
       <c r="D2" s="48"/>
@@ -4956,19 +4963,19 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="158" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="163" t="s">
-        <v>721</v>
-      </c>
-      <c r="B18" s="164"/>
-      <c r="C18" s="164"/>
-      <c r="D18" s="164"/>
-      <c r="E18" s="164"/>
-      <c r="F18" s="164"/>
-      <c r="G18" s="165"/>
+      <c r="A18" s="169" t="s">
+        <v>718</v>
+      </c>
+      <c r="B18" s="170"/>
+      <c r="C18" s="170"/>
+      <c r="D18" s="170"/>
+      <c r="E18" s="170"/>
+      <c r="F18" s="170"/>
+      <c r="G18" s="171"/>
       <c r="L18"/>
     </row>
   </sheetData>
@@ -5444,11 +5451,11 @@
         <v>16</v>
       </c>
       <c r="E2" s="8">
-        <f t="shared" ref="E2:E12" si="0">QUOTIENT(D2+7,8)</f>
+        <f t="shared" ref="E2:E3" si="0">QUOTIENT(D2+7,8)</f>
         <v>2</v>
       </c>
       <c r="F2" s="8">
-        <f t="shared" ref="F2:F12" si="1">QUOTIENT(E2+1,2)</f>
+        <f t="shared" ref="F2:F3" si="1">QUOTIENT(E2+1,2)</f>
         <v>1</v>
       </c>
       <c r="G2" s="16" t="s">
@@ -5458,7 +5465,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="145" t="str">
-        <f t="shared" ref="A3:A13" si="2">DEC2HEX(HEX2DEC(A2)+F2)</f>
+        <f t="shared" ref="A3:A8" si="2">DEC2HEX(HEX2DEC(A2)+F2)</f>
         <v>3E1</v>
       </c>
       <c r="B3" s="8" t="s">
@@ -5533,7 +5540,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="H5" s="18" t="s">
         <v>27</v>
@@ -5562,7 +5569,7 @@
         <v>4</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="H6" s="20" t="s">
         <v>29</v>
@@ -5628,7 +5635,7 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="145" t="str">
-        <f t="shared" ref="A9:A12" si="5">DEC2HEX(HEX2DEC(A8)+F8)</f>
+        <f>DEC2HEX(HEX2DEC(A8)+F8)</f>
         <v>3F2</v>
       </c>
       <c r="B9" s="18" t="s">
@@ -5641,11 +5648,11 @@
         <v>4</v>
       </c>
       <c r="E9" s="18">
-        <f t="shared" ref="E9:E11" si="6">QUOTIENT(D9+7,8)</f>
+        <f t="shared" ref="E9:E12" si="5">QUOTIENT(D9+7,8)</f>
         <v>1</v>
       </c>
       <c r="F9" s="18">
-        <f t="shared" ref="F9:F11" si="7">QUOTIENT(E9+1,2)</f>
+        <f t="shared" ref="F9:F12" si="6">QUOTIENT(E9+1,2)</f>
         <v>1</v>
       </c>
       <c r="G9" s="21" t="s">
@@ -5657,94 +5664,90 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="145" t="str">
+        <f>DEC2HEX(HEX2DEC(A9)+F9)</f>
+        <v>3F3</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="62" t="s">
+        <v>731</v>
+      </c>
+      <c r="D10" s="16">
+        <v>12</v>
+      </c>
+      <c r="E10" s="18">
         <f t="shared" si="5"/>
-        <v>3F3</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="62" t="s">
-        <v>322</v>
-      </c>
-      <c r="D10" s="16">
-        <v>32</v>
-      </c>
-      <c r="E10" s="18">
+        <v>2</v>
+      </c>
+      <c r="F10" s="18">
         <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="F10" s="18">
-        <f t="shared" si="7"/>
-        <v>2</v>
-      </c>
-      <c r="G10" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="H10" s="23" t="s">
-        <v>36</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="23"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="145" t="str">
+        <f>DEC2HEX(HEX2DEC(A9)+F9)</f>
+        <v>3F3</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="62" t="s">
+        <v>322</v>
+      </c>
+      <c r="D11" s="16">
+        <v>32</v>
+      </c>
+      <c r="E11" s="18">
         <f t="shared" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="F11" s="18">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="145" t="str">
+        <f t="shared" ref="A12" si="7">DEC2HEX(HEX2DEC(A11)+F11)</f>
         <v>3F5</v>
       </c>
-      <c r="B11" s="18" t="s">
-        <v>694</v>
-      </c>
-      <c r="C11" s="95" t="s">
-        <v>331</v>
-      </c>
-      <c r="D11" s="16">
-        <v>128</v>
-      </c>
-      <c r="E11" s="18">
+      <c r="B12" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="95" t="s">
+        <v>730</v>
+      </c>
+      <c r="D12" s="16">
+        <v>176</v>
+      </c>
+      <c r="E12" s="18">
+        <f t="shared" si="5"/>
+        <v>22</v>
+      </c>
+      <c r="F12" s="18">
         <f t="shared" si="6"/>
-        <v>16</v>
-      </c>
-      <c r="F11" s="18">
-        <f t="shared" si="7"/>
-        <v>8</v>
-      </c>
-      <c r="G11" s="16" t="s">
-        <v>699</v>
-      </c>
-      <c r="H11" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="148" t="str">
-        <f t="shared" si="5"/>
-        <v>3FD</v>
-      </c>
-      <c r="B12" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="62" t="s">
-        <v>700</v>
-      </c>
-      <c r="D12" s="24">
-        <v>48</v>
-      </c>
-      <c r="E12" s="24">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="F12" s="24">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="G12" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="H12" s="21" t="s">
-        <v>25</v>
-      </c>
+      <c r="H12" s="20"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="str">
-        <f t="shared" si="2"/>
+        <f>DEC2HEX(HEX2DEC(A12)+F12)</f>
         <v>400</v>
       </c>
       <c r="B13" s="13" t="s">
@@ -5753,14 +5756,14 @@
       <c r="C13" s="60"/>
       <c r="D13" s="12">
         <f>SUM(D2:D12)</f>
-        <v>500</v>
+        <v>512</v>
       </c>
       <c r="E13" s="12">
-        <f>SUM(E2:E12)</f>
-        <v>63</v>
+        <f>QUOTIENT(D13+7,8)</f>
+        <v>64</v>
       </c>
       <c r="F13" s="12">
-        <f>SUM(F2:F12)</f>
+        <f>QUOTIENT(E13+1,2)</f>
         <v>32</v>
       </c>
       <c r="G13" s="12"/>
@@ -5776,7 +5779,7 @@
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="8">
-        <f>F13*16</f>
+        <f>D13</f>
         <v>512</v>
       </c>
       <c r="E14" s="8">
@@ -5926,7 +5929,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="34" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="H4" s="16" t="s">
         <v>370</v>
@@ -6059,12 +6062,12 @@
         <v>334</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A9" s="119">
         <v>400</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>25</v>
+        <v>732</v>
       </c>
       <c r="C9" s="63">
         <v>8</v>
@@ -6081,7 +6084,7 @@
         <v>1</v>
       </c>
       <c r="G9" s="71" t="s">
-        <v>25</v>
+        <v>733</v>
       </c>
       <c r="H9" s="16" t="s">
         <v>370</v>
@@ -6405,7 +6408,7 @@
         <v>402</v>
       </c>
       <c r="B20" s="36" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C20" s="63">
         <v>14</v>
@@ -6422,7 +6425,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="34" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="H20" s="34"/>
       <c r="I20" s="19" t="s">
@@ -6567,7 +6570,7 @@
         <v>1</v>
       </c>
       <c r="G25" s="78" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="H25" s="58" t="s">
         <v>402</v>
@@ -7960,7 +7963,7 @@
         <v>344</v>
       </c>
       <c r="B71" s="28" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="C71" s="99">
         <v>7</v>
@@ -7977,7 +7980,7 @@
         <v>1</v>
       </c>
       <c r="G71" s="19" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="H71" s="58" t="s">
         <v>408</v>
@@ -7991,7 +7994,7 @@
         <v>344</v>
       </c>
       <c r="B72" s="29" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="C72" s="99">
         <v>6</v>
@@ -8008,7 +8011,7 @@
         <v>1</v>
       </c>
       <c r="G72" s="85" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="H72" s="58" t="s">
         <v>408</v>
@@ -8022,7 +8025,7 @@
         <v>344</v>
       </c>
       <c r="B73" s="29" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="C73" s="99">
         <v>5</v>
@@ -8039,7 +8042,7 @@
         <v>1</v>
       </c>
       <c r="G73" s="89" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="H73" s="58" t="s">
         <v>408</v>
@@ -8053,7 +8056,7 @@
         <v>344</v>
       </c>
       <c r="B74" s="29" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="C74" s="99">
         <v>4</v>
@@ -8070,7 +8073,7 @@
         <v>1</v>
       </c>
       <c r="G74" s="89" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="H74" s="58" t="s">
         <v>408</v>
@@ -8084,7 +8087,7 @@
         <v>344</v>
       </c>
       <c r="B75" s="29" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="C75" s="99">
         <v>3</v>
@@ -8101,7 +8104,7 @@
         <v>1</v>
       </c>
       <c r="G75" s="89" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="H75" s="58" t="s">
         <v>408</v>
@@ -8115,7 +8118,7 @@
         <v>344</v>
       </c>
       <c r="B76" s="29" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="C76" s="99">
         <v>2</v>
@@ -8132,7 +8135,7 @@
         <v>1</v>
       </c>
       <c r="G76" s="89" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="H76" s="58" t="s">
         <v>408</v>
@@ -8145,8 +8148,8 @@
       <c r="A77" s="119" t="s">
         <v>344</v>
       </c>
-      <c r="B77" s="171" t="s">
-        <v>706</v>
+      <c r="B77" s="167" t="s">
+        <v>703</v>
       </c>
       <c r="C77" s="63">
         <v>1</v>
@@ -8177,7 +8180,7 @@
         <v>344</v>
       </c>
       <c r="B78" s="81" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="C78" s="94">
         <v>0</v>
@@ -10415,7 +10418,7 @@
         <v>548</v>
       </c>
       <c r="H2" s="161" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="I2" s="143"/>
     </row>
@@ -10444,7 +10447,7 @@
         <v>549</v>
       </c>
       <c r="H3" s="161" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="I3" s="143"/>
     </row>
@@ -11022,7 +11025,7 @@
         <v>1</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>195</v>
@@ -12253,7 +12256,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>642</v>
@@ -13906,14 +13909,14 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="167" t="s">
+      <c r="A2" s="163" t="s">
         <v>565</v>
       </c>
-      <c r="B2" s="168" t="s">
-        <v>726</v>
-      </c>
-      <c r="C2" s="169" t="s">
-        <v>729</v>
+      <c r="B2" s="164" t="s">
+        <v>722</v>
+      </c>
+      <c r="C2" s="165" t="s">
+        <v>725</v>
       </c>
       <c r="D2" s="67">
         <v>5120</v>
@@ -13926,20 +13929,20 @@
         <f t="shared" ref="F2" si="1">QUOTIENT(E2+1,2)</f>
         <v>320</v>
       </c>
-      <c r="G2" s="170" t="s">
+      <c r="G2" s="166" t="s">
         <v>652</v>
       </c>
       <c r="H2" s="10"/>
     </row>
     <row r="3" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="167" t="s">
-        <v>730</v>
-      </c>
-      <c r="B3" s="168" t="s">
-        <v>727</v>
-      </c>
-      <c r="C3" s="169" t="s">
-        <v>729</v>
+      <c r="A3" s="163" t="s">
+        <v>726</v>
+      </c>
+      <c r="B3" s="164" t="s">
+        <v>723</v>
+      </c>
+      <c r="C3" s="165" t="s">
+        <v>725</v>
       </c>
       <c r="D3" s="67">
         <v>5120</v>
@@ -13952,20 +13955,20 @@
         <f t="shared" ref="F3:F4" si="3">QUOTIENT(E3+1,2)</f>
         <v>320</v>
       </c>
-      <c r="G3" s="170" t="s">
+      <c r="G3" s="166" t="s">
         <v>652</v>
       </c>
       <c r="H3" s="156"/>
     </row>
     <row r="4" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="167" t="s">
-        <v>731</v>
-      </c>
-      <c r="B4" s="168" t="s">
-        <v>728</v>
-      </c>
-      <c r="C4" s="169" t="s">
-        <v>729</v>
+      <c r="A4" s="163" t="s">
+        <v>727</v>
+      </c>
+      <c r="B4" s="164" t="s">
+        <v>724</v>
+      </c>
+      <c r="C4" s="165" t="s">
+        <v>725</v>
       </c>
       <c r="D4" s="67">
         <v>5120</v>
@@ -13978,20 +13981,20 @@
         <f t="shared" si="3"/>
         <v>320</v>
       </c>
-      <c r="G4" s="170" t="s">
+      <c r="G4" s="166" t="s">
         <v>652</v>
       </c>
       <c r="H4" s="156"/>
     </row>
     <row r="5" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="155" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="B5" s="157" t="s">
         <v>21</v>
       </c>
       <c r="C5" s="49" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="D5" s="8">
         <v>32768</v>
@@ -14004,8 +14007,8 @@
         <f t="shared" ref="F5" si="5">QUOTIENT(E5+1,2)</f>
         <v>2048</v>
       </c>
-      <c r="G5" s="166" t="s">
-        <v>704</v>
+      <c r="G5" s="162" t="s">
+        <v>701</v>
       </c>
       <c r="H5" s="156"/>
     </row>
@@ -15713,34 +15716,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="0358a91d-8923-4300-9035-92feb74d70aa">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="94916c3f-a887-466e-9071-419f2f5fc067" xsi:nil="true"/>
-    <TaxCatchAll xmlns="0358a91d-8923-4300-9035-92feb74d70aa" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="94916c3f-a887-466e-9071-419f2f5fc067">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB031FF8E1109D43B2BDF0F43F684A4E" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b896ebdbfa452e7a07541eac816e2062">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="94916c3f-a887-466e-9071-419f2f5fc067" xmlns:ns3="0358a91d-8923-4300-9035-92feb74d70aa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="556acc82b7336cf142ff4903a3ab7ecb" ns2:_="" ns3:_="">
     <xsd:import namespace="94916c3f-a887-466e-9071-419f2f5fc067"/>
@@ -15995,10 +15970,49 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="0358a91d-8923-4300-9035-92feb74d70aa">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="94916c3f-a887-466e-9071-419f2f5fc067" xsi:nil="true"/>
+    <TaxCatchAll xmlns="0358a91d-8923-4300-9035-92feb74d70aa" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="94916c3f-a887-466e-9071-419f2f5fc067">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06808489-AD29-49EF-A920-5725306266D8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AAF0E9-722A-46AD-84E0-1D9BE67AFFE4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="94916c3f-a887-466e-9071-419f2f5fc067"/>
+    <ds:schemaRef ds:uri="0358a91d-8923-4300-9035-92feb74d70aa"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -16021,20 +16035,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AAF0E9-722A-46AD-84E0-1D9BE67AFFE4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06808489-AD29-49EF-A920-5725306266D8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="94916c3f-a887-466e-9071-419f2f5fc067"/>
-    <ds:schemaRef ds:uri="0358a91d-8923-4300-9035-92feb74d70aa"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>